<commit_message>
config: 切换至 rewrite_existing pro 模式 + main.tex 添加硬件环境描述
- paper_spine_config.json: workflow->rewrite_existing, tier->pro, 更新目标名称/动因/特殊要求
- main.tex: 增加实验硬件环境段落，移除基金致谢行
- 清理已迁移的 final_paper_en 目录
- traffic_full/ 分析脚本修改
- final_paper_zh/main.tex 同步更新

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lane_coeffs.xlsx
+++ b/lane_coeffs.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="13380"/>
+    <workbookView windowWidth="29868" windowHeight="13380" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="85">
   <si>
     <t>where</t>
   </si>
@@ -320,6 +320,75 @@
 [2.3167669180504765e-13,-1.4722473199667758e-10,-9.454388404139244e-08,6.37479619002212e-05,-0.013023984224198938,31.950575625875086],
 [-4.453838475745655e-13,4.958640659657742e-10,-3.0483436242494034e-07,9.264582929543136e-05,-0.01451484937267032,35.671905452690936],
 [-4.453838475745655e-13,4.958640659657742e-10,-3.0483436242494034e-07,9.264582929543136e-05,-0.01451484937267032,39.52190545269094]</t>
+  </si>
+  <si>
+    <t>期刊名</t>
+  </si>
+  <si>
+    <t>分区</t>
+  </si>
+  <si>
+    <t>IF</t>
+  </si>
+  <si>
+    <t>审稿时间</t>
+  </si>
+  <si>
+    <t>OA</t>
+  </si>
+  <si>
+    <t>journal of traffic and transportation engineering(jtte)</t>
+  </si>
+  <si>
+    <t>中科院2区 / JCR Q1</t>
+  </si>
+  <si>
+    <t>6.8-9.3</t>
+  </si>
+  <si>
+    <t>平均15周</t>
+  </si>
+  <si>
+    <t>OA/无版面费</t>
+  </si>
+  <si>
+    <t>Accident Analysis &amp; Prevention（AAP）</t>
+  </si>
+  <si>
+    <t>中科院1区 / JCR Q1</t>
+  </si>
+  <si>
+    <t>参考5个月</t>
+  </si>
+  <si>
+    <t>非OA</t>
+  </si>
+  <si>
+    <t>Journal of Intelligent Transportation Systems（JITS）</t>
+  </si>
+  <si>
+    <t>中科院3区 / JCR Q2</t>
+  </si>
+  <si>
+    <t>3-6个月</t>
+  </si>
+  <si>
+    <t>Transportmetrica A: Transport Science</t>
+  </si>
+  <si>
+    <t>3.1-3.6</t>
+  </si>
+  <si>
+    <t>整体2-3月</t>
+  </si>
+  <si>
+    <t>Transportation Research Record（TRR）</t>
+  </si>
+  <si>
+    <t>中科院4区 / JCR Q3</t>
+  </si>
+  <si>
+    <t>三个月</t>
   </si>
 </sst>
 </file>
@@ -332,21 +401,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -819,152 +874,146 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1431,7 +1480,7 @@
       </c>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="2">
@@ -1460,7 +1509,7 @@
       </c>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B7" s="2">
@@ -1487,7 +1536,7 @@
       </c>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B8" s="2">
@@ -1516,7 +1565,7 @@
       </c>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B9" s="2">
@@ -1543,7 +1592,7 @@
       </c>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B10" s="2">
@@ -1571,7 +1620,7 @@
       </c>
     </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B11" s="2">
@@ -1598,7 +1647,7 @@
       </c>
     </row>
     <row r="12" spans="1:9">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B12" s="2">
@@ -1627,7 +1676,7 @@
       </c>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B13" s="2">
@@ -1656,7 +1705,7 @@
       </c>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B14" s="2">
@@ -1680,12 +1729,12 @@
       <c r="H14" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" s="4" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:9">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B15" s="2">
@@ -1707,12 +1756,12 @@
         <v>409</v>
       </c>
       <c r="H15" s="2"/>
-      <c r="I15" s="5" t="s">
+      <c r="I15" s="4" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:9">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B16" s="2">
@@ -1734,7 +1783,7 @@
         <v>735</v>
       </c>
       <c r="H16" s="2"/>
-      <c r="I16" s="6" t="s">
+      <c r="I16" s="4" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1748,9 +1797,119 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
-  <sheetData/>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="5" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="55.7777777777778" customWidth="1"/>
+    <col min="2" max="2" width="18.6666666666667" customWidth="1"/>
+    <col min="3" max="3" width="8.66666666666667" customWidth="1"/>
+    <col min="4" max="4" width="9.66666666666667" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3">
+        <v>6.2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4">
+        <v>2.8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6">
+        <v>1.8</v>
+      </c>
+      <c r="D6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>

</xml_diff>